<commit_message>
fix: apply gray background only to weekend and holiday rows in Excel and PDF exports
</commit_message>
<xml_diff>
--- a/public/templates/template_timesheet.xlsx
+++ b/public/templates/template_timesheet.xlsx
@@ -418,7 +418,7 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="21" fontId="8" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -929,11 +929,11 @@
     <col min="18" max="18" width="27.14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="17:18" x14ac:dyDescent="0.25">
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
     </row>
-    <row r="2" ht="24.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" ht="24.75" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -955,7 +955,7 @@
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
     </row>
-    <row r="3" ht="18.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" ht="18.75" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
@@ -977,7 +977,7 @@
       <c r="Q3" s="1"/>
       <c r="R3" s="1"/>
     </row>
-    <row r="4" ht="18.75" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" ht="18.75" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
@@ -999,7 +999,7 @@
       <c r="Q4" s="1"/>
       <c r="R4" s="1"/>
     </row>
-    <row r="5" ht="17.25" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" ht="17.25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
         <v>6</v>
       </c>
@@ -1021,7 +1021,7 @@
       <c r="Q5" s="1"/>
       <c r="R5" s="1"/>
     </row>
-    <row r="6" ht="17.25" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" ht="17.25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
         <v>8</v>
       </c>
@@ -1042,7 +1042,7 @@
       <c r="Q6" s="1"/>
       <c r="R6" s="1"/>
     </row>
-    <row r="7" ht="17.25" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" ht="17.25" customHeight="1" spans="4:18" x14ac:dyDescent="0.25">
       <c r="D7" s="13"/>
       <c r="E7" s="13"/>
       <c r="F7" s="14"/>
@@ -1060,7 +1060,7 @@
       <c r="Q7" s="19"/>
       <c r="R7" s="19"/>
     </row>
-    <row r="8" ht="17.25" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" ht="17.25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B8" s="20" t="s">
         <v>12</v>
       </c>
@@ -1097,7 +1097,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" ht="23.25" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" ht="23.25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B9" s="20"/>
       <c r="C9" s="22" t="s">
         <v>21</v>
@@ -1132,7 +1132,7 @@
       <c r="Q9" s="26"/>
       <c r="R9" s="26"/>
     </row>
-    <row r="10" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B10" s="28"/>
       <c r="C10" s="29"/>
       <c r="D10" s="29"/>
@@ -1151,7 +1151,7 @@
       <c r="Q10" s="32"/>
       <c r="R10" s="32"/>
     </row>
-    <row r="11" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B11" s="28"/>
       <c r="C11" s="29"/>
       <c r="D11" s="29"/>
@@ -1170,7 +1170,7 @@
       <c r="Q11" s="32"/>
       <c r="R11" s="32"/>
     </row>
-    <row r="12" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B12" s="28"/>
       <c r="C12" s="29"/>
       <c r="D12" s="29"/>
@@ -1189,7 +1189,7 @@
       <c r="Q12" s="32"/>
       <c r="R12" s="32"/>
     </row>
-    <row r="13" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="13" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B13" s="28"/>
       <c r="C13" s="29"/>
       <c r="D13" s="29"/>
@@ -1208,7 +1208,7 @@
       <c r="Q13" s="32"/>
       <c r="R13" s="32"/>
     </row>
-    <row r="14" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B14" s="28"/>
       <c r="C14" s="29"/>
       <c r="D14" s="29"/>
@@ -1227,7 +1227,7 @@
       <c r="Q14" s="32"/>
       <c r="R14" s="32"/>
     </row>
-    <row r="15" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B15" s="28"/>
       <c r="C15" s="29"/>
       <c r="D15" s="29"/>
@@ -1246,7 +1246,7 @@
       <c r="Q15" s="32"/>
       <c r="R15" s="32"/>
     </row>
-    <row r="16" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B16" s="28"/>
       <c r="C16" s="29"/>
       <c r="D16" s="29"/>
@@ -1265,7 +1265,7 @@
       <c r="Q16" s="32"/>
       <c r="R16" s="32"/>
     </row>
-    <row r="17" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="17" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B17" s="28"/>
       <c r="C17" s="29"/>
       <c r="D17" s="29"/>
@@ -1284,7 +1284,7 @@
       <c r="Q17" s="32"/>
       <c r="R17" s="32"/>
     </row>
-    <row r="18" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="18" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B18" s="28"/>
       <c r="C18" s="29"/>
       <c r="D18" s="29"/>
@@ -1303,7 +1303,7 @@
       <c r="Q18" s="32"/>
       <c r="R18" s="32"/>
     </row>
-    <row r="19" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="19" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B19" s="28"/>
       <c r="C19" s="29"/>
       <c r="D19" s="29"/>
@@ -1322,7 +1322,7 @@
       <c r="Q19" s="32"/>
       <c r="R19" s="32"/>
     </row>
-    <row r="20" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="20" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B20" s="28"/>
       <c r="C20" s="29"/>
       <c r="D20" s="29"/>
@@ -1341,7 +1341,7 @@
       <c r="Q20" s="32"/>
       <c r="R20" s="32"/>
     </row>
-    <row r="21" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B21" s="28"/>
       <c r="C21" s="29"/>
       <c r="D21" s="29"/>
@@ -1360,7 +1360,7 @@
       <c r="Q21" s="32"/>
       <c r="R21" s="32"/>
     </row>
-    <row r="22" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="22" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B22" s="28"/>
       <c r="C22" s="29"/>
       <c r="D22" s="29"/>
@@ -1379,7 +1379,7 @@
       <c r="Q22" s="32"/>
       <c r="R22" s="32"/>
     </row>
-    <row r="23" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="23" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B23" s="28"/>
       <c r="C23" s="29"/>
       <c r="D23" s="29"/>
@@ -1398,7 +1398,7 @@
       <c r="Q23" s="32"/>
       <c r="R23" s="32"/>
     </row>
-    <row r="24" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="24" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B24" s="28"/>
       <c r="C24" s="29"/>
       <c r="D24" s="29"/>
@@ -1417,7 +1417,7 @@
       <c r="Q24" s="32"/>
       <c r="R24" s="32"/>
     </row>
-    <row r="25" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="25" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B25" s="28"/>
       <c r="C25" s="29"/>
       <c r="D25" s="29"/>
@@ -1436,7 +1436,7 @@
       <c r="Q25" s="32"/>
       <c r="R25" s="32"/>
     </row>
-    <row r="26" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="26" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B26" s="28"/>
       <c r="C26" s="29"/>
       <c r="D26" s="29"/>
@@ -1455,7 +1455,7 @@
       <c r="Q26" s="32"/>
       <c r="R26" s="32"/>
     </row>
-    <row r="27" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="27" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B27" s="28"/>
       <c r="C27" s="29"/>
       <c r="D27" s="29"/>
@@ -1474,7 +1474,7 @@
       <c r="Q27" s="32"/>
       <c r="R27" s="32"/>
     </row>
-    <row r="28" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="28" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B28" s="28"/>
       <c r="C28" s="29"/>
       <c r="D28" s="29"/>
@@ -1493,7 +1493,7 @@
       <c r="Q28" s="32"/>
       <c r="R28" s="32"/>
     </row>
-    <row r="29" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="29" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B29" s="28"/>
       <c r="C29" s="29"/>
       <c r="D29" s="29"/>
@@ -1512,7 +1512,7 @@
       <c r="Q29" s="32"/>
       <c r="R29" s="32"/>
     </row>
-    <row r="30" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="30" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B30" s="28"/>
       <c r="C30" s="29"/>
       <c r="D30" s="29"/>
@@ -1531,7 +1531,7 @@
       <c r="Q30" s="32"/>
       <c r="R30" s="32"/>
     </row>
-    <row r="31" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="31" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B31" s="28"/>
       <c r="C31" s="29"/>
       <c r="D31" s="29"/>
@@ -1550,7 +1550,7 @@
       <c r="Q31" s="32"/>
       <c r="R31" s="32"/>
     </row>
-    <row r="32" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="32" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B32" s="28"/>
       <c r="C32" s="29"/>
       <c r="D32" s="29"/>
@@ -1569,7 +1569,7 @@
       <c r="Q32" s="32"/>
       <c r="R32" s="32"/>
     </row>
-    <row r="33" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B33" s="28"/>
       <c r="C33" s="29"/>
       <c r="D33" s="29"/>
@@ -1588,7 +1588,7 @@
       <c r="Q33" s="32"/>
       <c r="R33" s="32"/>
     </row>
-    <row r="34" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B34" s="28"/>
       <c r="C34" s="29"/>
       <c r="D34" s="29"/>
@@ -1607,7 +1607,7 @@
       <c r="Q34" s="32"/>
       <c r="R34" s="32"/>
     </row>
-    <row r="35" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B35" s="28"/>
       <c r="C35" s="29"/>
       <c r="D35" s="29"/>
@@ -1626,7 +1626,7 @@
       <c r="Q35" s="32"/>
       <c r="R35" s="32"/>
     </row>
-    <row r="36" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B36" s="28"/>
       <c r="C36" s="29"/>
       <c r="D36" s="29"/>
@@ -1645,7 +1645,7 @@
       <c r="Q36" s="32"/>
       <c r="R36" s="32"/>
     </row>
-    <row r="37" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B37" s="28"/>
       <c r="C37" s="29"/>
       <c r="D37" s="29"/>
@@ -1664,7 +1664,7 @@
       <c r="Q37" s="32"/>
       <c r="R37" s="32"/>
     </row>
-    <row r="38" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B38" s="28"/>
       <c r="C38" s="29"/>
       <c r="D38" s="29"/>
@@ -1683,7 +1683,7 @@
       <c r="Q38" s="32"/>
       <c r="R38" s="32"/>
     </row>
-    <row r="39" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B39" s="28"/>
       <c r="C39" s="29"/>
       <c r="D39" s="29"/>
@@ -1702,7 +1702,7 @@
       <c r="Q39" s="32"/>
       <c r="R39" s="32"/>
     </row>
-    <row r="40" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="40" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B40" s="28"/>
       <c r="C40" s="29"/>
       <c r="D40" s="29"/>
@@ -1721,7 +1721,7 @@
       <c r="Q40" s="32"/>
       <c r="R40" s="32"/>
     </row>
-    <row r="41" ht="15" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="41" ht="15" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B41" s="34"/>
       <c r="C41" s="34"/>
       <c r="D41" s="34"/>
@@ -1752,7 +1752,7 @@
       <c r="Q41" s="32"/>
       <c r="R41" s="32"/>
     </row>
-    <row r="42" ht="10" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="42" ht="10" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
@@ -1771,7 +1771,7 @@
       <c r="Q42" s="1"/>
       <c r="R42" s="1"/>
     </row>
-    <row r="43" ht="10.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" ht="10.5" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B43" s="39" t="s">
         <v>29</v>
       </c>
@@ -1824,7 +1824,7 @@
       <c r="Q44" s="38"/>
       <c r="R44" s="38"/>
     </row>
-    <row r="45" ht="18" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="45" ht="18" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B45" s="42"/>
       <c r="C45" s="42"/>
       <c r="D45" s="42"/>
@@ -1843,7 +1843,7 @@
       <c r="Q45" s="38"/>
       <c r="R45" s="38"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="46" ht="16.5" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B46" s="42"/>
       <c r="C46" s="42"/>
       <c r="D46" s="42"/>
@@ -1862,7 +1862,7 @@
       <c r="Q46" s="38"/>
       <c r="R46" s="38"/>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B47" s="42"/>
       <c r="C47" s="42"/>
       <c r="D47" s="42"/>
@@ -1881,7 +1881,7 @@
       <c r="Q47" s="38"/>
       <c r="R47" s="38"/>
     </row>
-    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B48" s="42"/>
       <c r="C48" s="42"/>
       <c r="D48" s="42"/>
@@ -1900,7 +1900,7 @@
       <c r="Q48" s="38"/>
       <c r="R48" s="38"/>
     </row>
-    <row r="49" ht="14.25" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="49" ht="14.25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B49" s="45" t="s">
         <v>36</v>
       </c>
@@ -1927,7 +1927,7 @@
       <c r="Q49" s="38"/>
       <c r="R49" s="38"/>
     </row>
-    <row r="50" ht="14.25" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="50" ht="14.25" customHeight="1" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B50" s="48" t="s">
         <v>40</v>
       </c>

</xml_diff>